<commit_message>
Weekly Premier League data update: 2026-09-17
</commit_message>
<xml_diff>
--- a/data/premier-league_xg_report.xlsx
+++ b/data/premier-league_xg_report.xlsx
@@ -9621,19 +9621,19 @@
         <v>1.33</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>2.08</v>
+        <v>1.99</v>
       </c>
       <c r="I5" s="10" t="n">
         <v>0.88</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.59</v>
+        <v>0.5</v>
       </c>
       <c r="K5" s="10" t="n">
         <v>-0.45</v>
       </c>
       <c r="L5" s="10" t="n">
-        <v>0.34</v>
+        <v>0.32</v>
       </c>
       <c r="M5" s="10" t="n">
         <v>-0.08</v>
@@ -9862,16 +9862,16 @@
         <v>2</v>
       </c>
       <c r="E24" s="18" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
       <c r="F24" s="18" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
       <c r="G24" s="18" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="25">
@@ -9918,16 +9918,16 @@
         <v>3</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="F26" s="20" t="n">
         <v>0.43</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="H26" s="20" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>
@@ -12416,19 +12416,19 @@
         <v>0.88</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>2.08</v>
+        <v>1.99</v>
       </c>
       <c r="J5" s="10" t="n">
         <v>-0.45</v>
       </c>
       <c r="K5" s="10" t="n">
-        <v>0.59</v>
+        <v>0.5</v>
       </c>
       <c r="L5" s="10" t="n">
         <v>-0.47</v>
       </c>
       <c r="M5" s="10" t="n">
-        <v>0.29</v>
+        <v>0.27</v>
       </c>
       <c r="N5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -12682,16 +12682,16 @@
         <v>4</v>
       </c>
       <c r="E25" s="18" t="n">
-        <v>-0.61</v>
+        <v>-0.57</v>
       </c>
       <c r="F25" s="18" t="n">
-        <v>-0.61</v>
+        <v>-0.57</v>
       </c>
       <c r="G25" s="18" t="n">
-        <v>-0.51</v>
+        <v>-0.55</v>
       </c>
       <c r="H25" s="18" t="n">
-        <v>-0.51</v>
+        <v>-0.55</v>
       </c>
     </row>
     <row r="26">
@@ -12710,16 +12710,16 @@
         <v>8</v>
       </c>
       <c r="E26" s="20" t="n">
-        <v>-0.76</v>
+        <v>-0.74</v>
       </c>
       <c r="F26" s="20" t="n">
-        <v>-0.91</v>
+        <v>-0.86</v>
       </c>
       <c r="G26" s="20" t="n">
-        <v>-0.17</v>
+        <v>-0.2</v>
       </c>
       <c r="H26" s="20" t="n">
-        <v>-0.45</v>
+        <v>-0.49</v>
       </c>
     </row>
   </sheetData>
@@ -16153,118 +16153,118 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Leeds United</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="B5" s="8">
-        <f>'Leeds United'!$E$8</f>
+        <f>'Fulham'!$E$8</f>
         <v/>
       </c>
       <c r="C5" s="8">
-        <f>'Leeds United'!$E$9</f>
+        <f>'Fulham'!$E$9</f>
         <v/>
       </c>
       <c r="D5" s="8">
-        <f>'Leeds United'!$E$10</f>
+        <f>'Fulham'!$E$10</f>
         <v/>
       </c>
       <c r="E5" s="10">
-        <f>'Leeds United'!$E$11</f>
+        <f>'Fulham'!$E$11</f>
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>'Leeds United'!$E$12</f>
+        <f>'Fulham'!$E$12</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>'Leeds United'!$E$13</f>
+        <f>'Fulham'!$E$13</f>
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>'Leeds United'!$E$14</f>
+        <f>'Fulham'!$E$14</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>'Leeds United'!$E$15</f>
+        <f>'Fulham'!$E$15</f>
         <v/>
       </c>
       <c r="J5" s="10">
-        <f>'Leeds United'!$E$16</f>
+        <f>'Fulham'!$E$16</f>
         <v/>
       </c>
       <c r="K5" s="10">
-        <f>'Leeds United'!$E$17</f>
+        <f>'Fulham'!$E$17</f>
         <v/>
       </c>
       <c r="L5" s="10">
-        <f>'Leeds United'!$E$18</f>
+        <f>'Fulham'!$E$18</f>
         <v/>
       </c>
       <c r="M5" s="10">
-        <f>'Leeds United'!$E$19</f>
+        <f>'Fulham'!$E$19</f>
         <v/>
       </c>
       <c r="N5" s="10">
-        <f>'Leeds United'!$E$20</f>
+        <f>'Fulham'!$E$20</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="B6" s="6">
-        <f>'Fulham'!$E$8</f>
+        <f>'Leeds United'!$E$8</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>'Fulham'!$E$9</f>
+        <f>'Leeds United'!$E$9</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>'Fulham'!$E$10</f>
+        <f>'Leeds United'!$E$10</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>'Fulham'!$E$11</f>
+        <f>'Leeds United'!$E$11</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>'Fulham'!$E$12</f>
+        <f>'Leeds United'!$E$12</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>'Fulham'!$E$13</f>
+        <f>'Leeds United'!$E$13</f>
         <v/>
       </c>
       <c r="H6" s="9">
-        <f>'Fulham'!$E$14</f>
+        <f>'Leeds United'!$E$14</f>
         <v/>
       </c>
       <c r="I6" s="9">
-        <f>'Fulham'!$E$15</f>
+        <f>'Leeds United'!$E$15</f>
         <v/>
       </c>
       <c r="J6" s="9">
-        <f>'Fulham'!$E$16</f>
+        <f>'Leeds United'!$E$16</f>
         <v/>
       </c>
       <c r="K6" s="9">
-        <f>'Fulham'!$E$17</f>
+        <f>'Leeds United'!$E$17</f>
         <v/>
       </c>
       <c r="L6" s="9">
-        <f>'Fulham'!$E$18</f>
+        <f>'Leeds United'!$E$18</f>
         <v/>
       </c>
       <c r="M6" s="9">
-        <f>'Fulham'!$E$19</f>
+        <f>'Leeds United'!$E$19</f>
         <v/>
       </c>
       <c r="N6" s="9">
-        <f>'Fulham'!$E$20</f>
+        <f>'Leeds United'!$E$20</f>
         <v/>
       </c>
     </row>
@@ -17497,16 +17497,16 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0.43</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>0.43</v>
@@ -17772,10 +17772,10 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>-0.76</v>
+        <v>-0.74</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>-0.91</v>
+        <v>-0.86</v>
       </c>
       <c r="D20" s="10" t="n">
         <v>-0.91</v>
@@ -17784,10 +17784,10 @@
         <v>-0.91</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>-0.61</v>
+        <v>-0.57</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>-0.61</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="21">
@@ -18598,54 +18598,54 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Leeds United</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="B5" s="12">
-        <f>'Leeds United'!$E$15</f>
+        <f>'Fulham'!$E$15</f>
         <v/>
       </c>
       <c r="C5" s="9">
-        <f>'Leeds United'!$N$2</f>
+        <f>'Fulham'!$N$2</f>
         <v/>
       </c>
       <c r="D5" s="9">
-        <f>'Leeds United'!$N$3</f>
+        <f>'Fulham'!$N$3</f>
         <v/>
       </c>
       <c r="E5" s="9">
-        <f>'Leeds United'!$N$4</f>
+        <f>'Fulham'!$N$4</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>'Leeds United'!$N$5</f>
+        <f>'Fulham'!$N$5</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="B6" s="12">
-        <f>'Fulham'!$E$15</f>
+        <f>'Leeds United'!$E$15</f>
         <v/>
       </c>
       <c r="C6" s="9">
-        <f>'Fulham'!$N$2</f>
+        <f>'Leeds United'!$N$2</f>
         <v/>
       </c>
       <c r="D6" s="9">
-        <f>'Fulham'!$N$3</f>
+        <f>'Leeds United'!$N$3</f>
         <v/>
       </c>
       <c r="E6" s="9">
-        <f>'Fulham'!$N$4</f>
+        <f>'Leeds United'!$N$4</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>'Fulham'!$N$5</f>
+        <f>'Leeds United'!$N$5</f>
         <v/>
       </c>
     </row>
@@ -19160,33 +19160,33 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Leeds United</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>0.41</v>
+        <v>0.27</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>-0.24</v>
+        <v>-0.37</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>1.05</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>0.27</v>
+        <v>0.36</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>-0.37</v>
+        <v>-0.24</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>0.91</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="7">
@@ -19535,33 +19535,33 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Leeds United</t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>0.43</v>
+        <v>-0.08</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>0.04</v>
+        <v>-0.88</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>0.83</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Fulham</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>-0.08</v>
+        <v>0.43</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>-0.88</v>
+        <v>0.04</v>
       </c>
       <c r="D6" s="9" t="n">
-        <v>0.73</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="7">
@@ -19747,13 +19747,13 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>-0.61</v>
+        <v>-0.57</v>
       </c>
       <c r="C18" s="9" t="n">
         <v>-0.18</v>
       </c>
       <c r="D18" s="9" t="n">
-        <v>-1.05</v>
+        <v>-0.96</v>
       </c>
     </row>
     <row r="19">
@@ -20036,54 +20036,54 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Leeds United</t>
+          <t>Ipswich</t>
         </is>
       </c>
       <c r="B8" s="12">
-        <f>'Leeds United'!$E$17</f>
+        <f>'Ipswich'!$E$17</f>
         <v/>
       </c>
       <c r="C8" s="9">
-        <f>'Leeds United'!$O$2</f>
+        <f>'Ipswich'!$O$2</f>
         <v/>
       </c>
       <c r="D8" s="9">
-        <f>'Leeds United'!$O$3</f>
+        <f>'Ipswich'!$O$3</f>
         <v/>
       </c>
       <c r="E8" s="9">
-        <f>'Leeds United'!$O$4</f>
+        <f>'Ipswich'!$O$4</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>'Leeds United'!$O$5</f>
+        <f>'Ipswich'!$O$5</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Ipswich</t>
+          <t>Leeds United</t>
         </is>
       </c>
       <c r="B9" s="12">
-        <f>'Ipswich'!$E$17</f>
+        <f>'Leeds United'!$E$17</f>
         <v/>
       </c>
       <c r="C9" s="9">
-        <f>'Ipswich'!$O$2</f>
+        <f>'Leeds United'!$O$2</f>
         <v/>
       </c>
       <c r="D9" s="9">
-        <f>'Ipswich'!$O$3</f>
+        <f>'Leeds United'!$O$3</f>
         <v/>
       </c>
       <c r="E9" s="9">
-        <f>'Ipswich'!$O$4</f>
+        <f>'Leeds United'!$O$4</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>'Ipswich'!$O$5</f>
+        <f>'Leeds United'!$O$5</f>
         <v/>
       </c>
     </row>
@@ -20198,54 +20198,54 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Newcastle United</t>
+          <t>Nottingham Forest</t>
         </is>
       </c>
       <c r="B14" s="12">
-        <f>'Newcastle United'!$E$17</f>
+        <f>'Nottingham Forest'!$E$17</f>
         <v/>
       </c>
       <c r="C14" s="9">
-        <f>'Newcastle United'!$O$2</f>
+        <f>'Nottingham Forest'!$O$2</f>
         <v/>
       </c>
       <c r="D14" s="9">
-        <f>'Newcastle United'!$O$3</f>
+        <f>'Nottingham Forest'!$O$3</f>
         <v/>
       </c>
       <c r="E14" s="9">
-        <f>'Newcastle United'!$O$4</f>
+        <f>'Nottingham Forest'!$O$4</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>'Newcastle United'!$O$5</f>
+        <f>'Nottingham Forest'!$O$5</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Nottingham Forest</t>
+          <t>Newcastle United</t>
         </is>
       </c>
       <c r="B15" s="12">
-        <f>'Nottingham Forest'!$E$17</f>
+        <f>'Newcastle United'!$E$17</f>
         <v/>
       </c>
       <c r="C15" s="9">
-        <f>'Nottingham Forest'!$O$2</f>
+        <f>'Newcastle United'!$O$2</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>'Nottingham Forest'!$O$3</f>
+        <f>'Newcastle United'!$O$3</f>
         <v/>
       </c>
       <c r="E15" s="9">
-        <f>'Nottingham Forest'!$O$4</f>
+        <f>'Newcastle United'!$O$4</f>
         <v/>
       </c>
       <c r="F15" s="9">
-        <f>'Nottingham Forest'!$O$5</f>
+        <f>'Newcastle United'!$O$5</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Weekly Premier League data update: 2026-10-06
</commit_message>
<xml_diff>
--- a/data/premier-league_xg_report.xlsx
+++ b/data/premier-league_xg_report.xlsx
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="B13" s="14" t="n">
-        <v>-0.26</v>
+        <v>-0.29</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>0.18</v>
@@ -1410,7 +1410,7 @@
         <v>-0.88</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>-0.08</v>
+        <v>-0.18</v>
       </c>
     </row>
     <row r="14">
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="B20" s="14" t="n">
-        <v>-0.8</v>
+        <v>-0.77</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>-3.2</v>
@@ -1956,7 +1956,7 @@
         <v>0.72</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>0.08</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="21">
@@ -3327,62 +3327,62 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="B18" s="14">
-        <f>'Tottenham Hotspur'!$E$30</f>
+        <f>'Aston Villa'!$E$30</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>'Tottenham Hotspur'!$V$2</f>
+        <f>'Aston Villa'!$V$2</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>'Tottenham Hotspur'!$V$3</f>
+        <f>'Aston Villa'!$V$3</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>'Tottenham Hotspur'!$V$4</f>
+        <f>'Aston Villa'!$V$4</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>'Tottenham Hotspur'!$V$5</f>
+        <f>'Aston Villa'!$V$5</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>'Tottenham Hotspur'!$V$6</f>
+        <f>'Aston Villa'!$V$6</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="B19" s="14">
-        <f>'Aston Villa'!$E$30</f>
+        <f>'Tottenham Hotspur'!$E$30</f>
         <v/>
       </c>
       <c r="C19" s="9">
-        <f>'Aston Villa'!$V$2</f>
+        <f>'Tottenham Hotspur'!$V$2</f>
         <v/>
       </c>
       <c r="D19" s="9">
-        <f>'Aston Villa'!$V$3</f>
+        <f>'Tottenham Hotspur'!$V$3</f>
         <v/>
       </c>
       <c r="E19" s="9">
-        <f>'Aston Villa'!$V$4</f>
+        <f>'Tottenham Hotspur'!$V$4</f>
         <v/>
       </c>
       <c r="F19" s="9">
-        <f>'Aston Villa'!$V$5</f>
+        <f>'Tottenham Hotspur'!$V$5</f>
         <v/>
       </c>
       <c r="G19" s="9">
-        <f>'Aston Villa'!$V$6</f>
+        <f>'Tottenham Hotspur'!$V$6</f>
         <v/>
       </c>
     </row>
@@ -3755,13 +3755,13 @@
         <v>-1.58</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>-0.19</v>
+        <v>-0.21</v>
       </c>
       <c r="P3" s="10" t="n">
         <v>-1.02</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>-0.31</v>
+        <v>-0.33</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -3843,7 +3843,7 @@
         <v>-0.78</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.32</v>
+        <v>-0.33</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -5090,31 +5090,31 @@
         <v>1.63</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>1.16</v>
+        <v>1.26</v>
       </c>
       <c r="I6" s="9" t="n">
         <v>1.56</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>-0.07000000000000001</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>-0.4</v>
+        <v>-0.38</v>
       </c>
       <c r="M6" s="9" t="n">
         <v>0.36</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.29</v>
+        <v>-0.19</v>
       </c>
       <c r="O6" s="9" t="n">
         <v>0.53</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>-0.37</v>
+        <v>-0.35</v>
       </c>
       <c r="Q6" s="9" t="n">
         <v>0.39</v>
@@ -5128,16 +5128,16 @@
         <v/>
       </c>
       <c r="T6" s="9" t="n">
-        <v>1.1</v>
+        <v>1.17</v>
       </c>
       <c r="U6" s="9" t="n">
         <v>1.05</v>
       </c>
       <c r="V6" s="9" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="W6" s="9" t="n">
-        <v>4.7</v>
+        <v>4.77</v>
       </c>
       <c r="X6" s="9" t="n">
         <v>6.34</v>
@@ -5485,16 +5485,16 @@
         <v>6</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>-0.8</v>
+        <v>-0.77</v>
       </c>
       <c r="F35" s="19" t="n">
-        <v>0.08</v>
+        <v>0.18</v>
       </c>
       <c r="G35" s="19" t="n">
-        <v>0.27</v>
+        <v>0.31</v>
       </c>
       <c r="H35" s="19" t="n">
-        <v>-0.06</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="36">
@@ -5513,16 +5513,16 @@
         <v>9</v>
       </c>
       <c r="E36" s="21" t="n">
-        <v>-0.76</v>
+        <v>-0.74</v>
       </c>
       <c r="F36" s="21" t="n">
-        <v>0.08</v>
+        <v>0.18</v>
       </c>
       <c r="G36" s="21" t="n">
-        <v>-0.04</v>
+        <v>-0.02</v>
       </c>
       <c r="H36" s="21" t="n">
-        <v>-0.06</v>
+        <v>0.04</v>
       </c>
     </row>
   </sheetData>
@@ -7000,13 +7000,13 @@
         <v>-0.84</v>
       </c>
       <c r="N2" s="9" t="n">
-        <v>2.62</v>
+        <v>2.6</v>
       </c>
       <c r="O2" s="9" t="n">
         <v>-0.44</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>2.62</v>
+        <v>2.6</v>
       </c>
       <c r="Q2" s="9" t="n">
         <v>-0.44</v>
@@ -7088,7 +7088,7 @@
         <v>-0.06</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>1.56</v>
+        <v>1.55</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>-0.25</v>
@@ -7170,7 +7170,7 @@
         <v>-0.17</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>-0.22</v>
@@ -7252,7 +7252,7 @@
         <v>0.35</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.37</v>
+        <v>0.36</v>
       </c>
       <c r="Q5" s="10" t="n">
         <v>-0.08</v>
@@ -8113,13 +8113,13 @@
         <v>2.24</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.84</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>2.24</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-0.84</v>
       </c>
       <c r="R2" s="9">
         <f>(H2-I2)-(F2-G2)</f>
@@ -8201,7 +8201,7 @@
         <v>1</v>
       </c>
       <c r="Q3" s="10" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
       <c r="R3" s="10">
         <f>(H3-I3)-(F3-G3)</f>
@@ -13734,7 +13734,7 @@
         <v>-0.1</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>-0.29</v>
+        <v>-0.32</v>
       </c>
       <c r="O5" s="10" t="n">
         <v>-0.48</v>
@@ -15875,13 +15875,13 @@
         <v>-1.04</v>
       </c>
       <c r="O4" s="9" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>-0.32</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="R4" s="9">
         <f>(H4-I4)-(F4-G4)</f>
@@ -15963,7 +15963,7 @@
         <v>-0.19</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.51</v>
+        <v>-0.52</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -16045,7 +16045,7 @@
         <v>-0.1</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>-0.43</v>
+        <v>-0.44</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -23656,13 +23656,13 @@
         <v>0.29</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>-1.14</v>
+        <v>-1.17</v>
       </c>
       <c r="O3" s="10" t="n">
         <v>0.01</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>-0.42</v>
+        <v>-0.44</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>0.93</v>
@@ -23744,7 +23744,7 @@
         <v>0.06</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.59</v>
+        <v>-0.6</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>0.64</v>
@@ -24848,13 +24848,13 @@
         <v>-0.42</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>-0.9</v>
+        <v>-0.92</v>
       </c>
       <c r="O4" s="9" t="n">
         <v>0.38</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="Q4" s="9" t="n">
         <v>-0.21</v>
@@ -24933,13 +24933,13 @@
         <v>0.93</v>
       </c>
       <c r="O5" s="10" t="n">
-        <v>-0.32</v>
+        <v>-0.35</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-0.23</v>
+        <v>-0.24</v>
       </c>
       <c r="R5" s="10">
         <f>(H5-I5)-(F5-G5)</f>
@@ -27217,31 +27217,31 @@
         <v>1.56</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>1.16</v>
+        <v>1.26</v>
       </c>
       <c r="J6" s="9" t="n">
         <v>-0.07000000000000001</v>
       </c>
       <c r="K6" s="9" t="n">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="L6" s="9" t="n">
         <v>-0.49</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>0.24</v>
+        <v>0.26</v>
       </c>
       <c r="N6" s="9" t="n">
         <v>-0.54</v>
       </c>
       <c r="O6" s="9" t="n">
-        <v>0.51</v>
+        <v>0.61</v>
       </c>
       <c r="P6" s="9" t="n">
         <v>-0.65</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.37</v>
+        <v>0.39</v>
       </c>
       <c r="R6" s="9">
         <f>(H6-I6)-(F6-G6)</f>
@@ -27252,16 +27252,16 @@
         <v/>
       </c>
       <c r="T6" s="9" t="n">
-        <v>1.65</v>
+        <v>1.58</v>
       </c>
       <c r="U6" s="9" t="n">
         <v>1.7</v>
       </c>
       <c r="V6" s="9" t="n">
-        <v>-0.05</v>
+        <v>-0.12</v>
       </c>
       <c r="W6" s="9" t="n">
-        <v>5.89</v>
+        <v>5.82</v>
       </c>
       <c r="X6" s="9" t="n">
         <v>7.49</v>
@@ -27581,13 +27581,13 @@
         <v>5</v>
       </c>
       <c r="E34" s="19" t="n">
-        <v>-0.26</v>
+        <v>-0.29</v>
       </c>
       <c r="F34" s="19" t="n">
-        <v>-0.08</v>
+        <v>-0.18</v>
       </c>
       <c r="G34" s="19" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.66</v>
       </c>
       <c r="H34" s="19" t="n">
         <v>-0.86</v>
@@ -27637,13 +27637,13 @@
         <v>8</v>
       </c>
       <c r="E36" s="21" t="n">
-        <v>-0.73</v>
+        <v>-0.75</v>
       </c>
       <c r="F36" s="21" t="n">
-        <v>-0.08</v>
+        <v>-0.18</v>
       </c>
       <c r="G36" s="21" t="n">
-        <v>-0.25</v>
+        <v>-0.23</v>
       </c>
       <c r="H36" s="21" t="n">
         <v>-0.66</v>
@@ -29479,19 +29479,19 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="C18" s="6">
-        <f>'Tottenham Hotspur'!$E$9</f>
+        <f>'Aston Villa'!$E$9</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>'Tottenham Hotspur'!$E$28</f>
+        <f>'Aston Villa'!$E$28</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>'Tottenham Hotspur'!$E$29</f>
+        <f>'Aston Villa'!$E$29</f>
         <v/>
       </c>
       <c r="F18" s="9">
@@ -29505,19 +29505,19 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="C19" s="8">
-        <f>'Aston Villa'!$E$9</f>
+        <f>'Tottenham Hotspur'!$E$9</f>
         <v/>
       </c>
       <c r="D19" s="10">
-        <f>'Aston Villa'!$E$28</f>
+        <f>'Tottenham Hotspur'!$E$28</f>
         <v/>
       </c>
       <c r="E19" s="10">
-        <f>'Aston Villa'!$E$29</f>
+        <f>'Tottenham Hotspur'!$E$29</f>
         <v/>
       </c>
       <c r="F19" s="10">
@@ -32282,25 +32282,25 @@
         <v>1.56</v>
       </c>
       <c r="I44" s="9" t="n">
-        <v>1.16</v>
+        <v>1.26</v>
       </c>
       <c r="J44" s="9" t="n">
         <v>-0.07000000000000001</v>
       </c>
       <c r="K44" s="9" t="n">
-        <v>0.01</v>
+        <v>0.11</v>
       </c>
       <c r="L44" s="9" t="n">
-        <v>-0.08</v>
+        <v>-0.18</v>
       </c>
       <c r="M44" s="9" t="n">
-        <v>-0.06</v>
+        <v>0.04</v>
       </c>
       <c r="N44" s="9" t="n">
-        <v>1.65</v>
+        <v>1.58</v>
       </c>
       <c r="O44" s="9" t="n">
-        <v>1.1</v>
+        <v>1.17</v>
       </c>
       <c r="P44" s="9" t="n">
         <v>1.7</v>
@@ -33241,51 +33241,51 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>-0.73</v>
+        <v>-0.74</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-0.08</v>
+        <v>0.18</v>
       </c>
       <c r="D19" s="9" t="n">
-        <v>-0.26</v>
+        <v>-0.7</v>
       </c>
       <c r="E19" s="9" t="n">
-        <v>-0.08</v>
+        <v>-0.7</v>
       </c>
       <c r="F19" s="9" t="n">
-        <v>-1.45</v>
+        <v>-0.77</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>-1.45</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>-0.76</v>
+        <v>-0.75</v>
       </c>
       <c r="C20" s="10" t="n">
-        <v>0.08</v>
+        <v>-0.18</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>-0.7</v>
+        <v>-0.29</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>-0.7</v>
+        <v>-0.18</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>-0.8</v>
+        <v>-1.45</v>
       </c>
       <c r="G20" s="10" t="n">
-        <v>0.08</v>
+        <v>-1.45</v>
       </c>
     </row>
     <row r="21">
@@ -33785,51 +33785,51 @@
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="B42" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C42" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D42" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C43" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E43" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="8" t="n">
         <v>3</v>
-      </c>
-      <c r="F43" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="G43" s="8" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="44">
@@ -34517,62 +34517,62 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Tottenham Hotspur</t>
+          <t>Aston Villa</t>
         </is>
       </c>
       <c r="B18" s="14">
-        <f>'Tottenham Hotspur'!$E$20</f>
+        <f>'Aston Villa'!$E$20</f>
         <v/>
       </c>
       <c r="C18" s="9">
-        <f>'Tottenham Hotspur'!$R$2</f>
+        <f>'Aston Villa'!$R$2</f>
         <v/>
       </c>
       <c r="D18" s="9">
-        <f>'Tottenham Hotspur'!$R$3</f>
+        <f>'Aston Villa'!$R$3</f>
         <v/>
       </c>
       <c r="E18" s="9">
-        <f>'Tottenham Hotspur'!$R$4</f>
+        <f>'Aston Villa'!$R$4</f>
         <v/>
       </c>
       <c r="F18" s="9">
-        <f>'Tottenham Hotspur'!$R$5</f>
+        <f>'Aston Villa'!$R$5</f>
         <v/>
       </c>
       <c r="G18" s="9">
-        <f>'Tottenham Hotspur'!$R$6</f>
+        <f>'Aston Villa'!$R$6</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Tottenham Hotspur</t>
         </is>
       </c>
       <c r="B19" s="14">
-        <f>'Aston Villa'!$E$20</f>
+        <f>'Tottenham Hotspur'!$E$20</f>
         <v/>
       </c>
       <c r="C19" s="9">
-        <f>'Aston Villa'!$R$2</f>
+        <f>'Tottenham Hotspur'!$R$2</f>
         <v/>
       </c>
       <c r="D19" s="9">
-        <f>'Aston Villa'!$R$3</f>
+        <f>'Tottenham Hotspur'!$R$3</f>
         <v/>
       </c>
       <c r="E19" s="9">
-        <f>'Aston Villa'!$R$4</f>
+        <f>'Tottenham Hotspur'!$R$4</f>
         <v/>
       </c>
       <c r="F19" s="9">
-        <f>'Aston Villa'!$R$5</f>
+        <f>'Tottenham Hotspur'!$R$5</f>
         <v/>
       </c>
       <c r="G19" s="9">
-        <f>'Aston Villa'!$R$6</f>
+        <f>'Tottenham Hotspur'!$R$6</f>
         <v/>
       </c>
     </row>

</xml_diff>